<commit_message>
feat: Add stations data CSV file with geographical and metadata information
</commit_message>
<xml_diff>
--- a/docs/importance_by_subtype.xlsx
+++ b/docs/importance_by_subtype.xlsx
@@ -517,19 +517,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.00226</v>
+        <v>0.00234</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00533</v>
+        <v>0.00566</v>
       </c>
       <c r="E2" t="n">
-        <v>0.000496</v>
+        <v>0.000487</v>
       </c>
       <c r="F2" t="n">
         <v>28</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0265</v>
+        <v>0.0273</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
@@ -551,15 +551,15 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>0/6/4</t>
+          <t>0/3/7</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>41.68</v>
+        <v>43.52</v>
       </c>
       <c r="N2" s="1" t="inlineStr">
         <is>
-          <t>4.52E-01</t>
+          <t>2.30E-01</t>
         </is>
       </c>
     </row>
@@ -575,19 +575,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.00107</v>
+        <v>0.00106</v>
       </c>
       <c r="D3" t="n">
-        <v>0.000341</v>
+        <v>0.000344</v>
       </c>
       <c r="E3" t="n">
-        <v>0.000513</v>
+        <v>0.000349</v>
       </c>
       <c r="F3" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00177</v>
+        <v>0.00164</v>
       </c>
       <c r="H3" t="n">
         <v>2</v>
@@ -609,11 +609,11 @@
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
-          <t>5/2/3</t>
+          <t>5/3/2</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>36.52</v>
+        <v>35.29</v>
       </c>
       <c r="N3" s="1" t="inlineStr">
         <is>
@@ -633,19 +633,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.000961</v>
+        <v>0.000922</v>
       </c>
       <c r="D4" t="n">
-        <v>0.000808</v>
+        <v>0.000697</v>
       </c>
       <c r="E4" t="n">
-        <v>0.000486</v>
+        <v>0.000507</v>
       </c>
       <c r="F4" t="n">
         <v>24</v>
       </c>
       <c r="G4" t="n">
-        <v>0.00377</v>
+        <v>0.00335</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
@@ -667,15 +667,15 @@
       </c>
       <c r="L4" s="1" t="inlineStr">
         <is>
-          <t>5/2/3</t>
+          <t>5/4/1</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>62.81</v>
+        <v>62.19</v>
       </c>
       <c r="N4" s="1" t="inlineStr">
         <is>
-          <t>2.51E-04</t>
+          <t>1.74E-04</t>
         </is>
       </c>
     </row>
@@ -691,19 +691,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.00345</v>
+        <v>0.00355</v>
       </c>
       <c r="D5" t="n">
-        <v>0.009039999999999999</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="E5" t="n">
         <v>0.000648</v>
       </c>
       <c r="F5" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0447</v>
+        <v>0.0448</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>40.29</v>
+        <v>40.06</v>
       </c>
       <c r="N5" s="1" t="inlineStr">
         <is>
@@ -749,19 +749,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.00128</v>
+        <v>0.00127</v>
       </c>
       <c r="D6" t="n">
-        <v>0.000801</v>
+        <v>0.000781</v>
       </c>
       <c r="E6" t="n">
-        <v>0.00042</v>
+        <v>0.000481</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00364</v>
+        <v>0.00347</v>
       </c>
       <c r="H6" t="n">
         <v>3</v>
@@ -783,15 +783,15 @@
       </c>
       <c r="L6" s="1" t="inlineStr">
         <is>
-          <t>3/4/1/2</t>
+          <t>3/4/2/1</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>44.32</v>
+        <v>44.61</v>
       </c>
       <c r="N6" s="1" t="inlineStr">
         <is>
-          <t>6.59E-01</t>
+          <t>6.18E-01</t>
         </is>
       </c>
     </row>
@@ -807,19 +807,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.000821</v>
+        <v>0.000807</v>
       </c>
       <c r="D7" t="n">
-        <v>0.000458</v>
+        <v>0.000449</v>
       </c>
       <c r="E7" t="n">
-        <v>0.000238</v>
+        <v>0.000251</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>0.00183</v>
+        <v>0.00178</v>
       </c>
       <c r="H7" t="n">
         <v>10</v>
@@ -836,20 +836,20 @@
       </c>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>0/1/1/5</t>
+          <t>0/1/0/6</t>
         </is>
       </c>
       <c r="L7" s="1" t="inlineStr">
         <is>
-          <t>2/2/3/3</t>
+          <t>2/2/2/4</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>71.48</v>
+        <v>72.48</v>
       </c>
       <c r="N7" s="1" t="inlineStr">
         <is>
-          <t>9.49E-04</t>
+          <t>5.75E-04</t>
         </is>
       </c>
     </row>
@@ -865,19 +865,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.000549</v>
+        <v>0.000537</v>
       </c>
       <c r="D8" t="n">
-        <v>0.000147</v>
+        <v>0.000135</v>
       </c>
       <c r="E8" t="n">
-        <v>0.00016</v>
+        <v>0.000152</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0011</v>
+        <v>0.00104</v>
       </c>
       <c r="H8" t="n">
         <v>4</v>
@@ -894,7 +894,7 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>0/0/5/2</t>
+          <t>0/0/6/1</t>
         </is>
       </c>
       <c r="L8" s="1" t="inlineStr">
@@ -903,11 +903,11 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>93.90000000000001</v>
+        <v>92.84</v>
       </c>
       <c r="N8" s="1" t="inlineStr">
         <is>
-          <t>1.28E-08</t>
+          <t>2.23E-08</t>
         </is>
       </c>
     </row>
@@ -923,49 +923,49 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.008449999999999999</v>
+        <v>0.00976</v>
       </c>
       <c r="D9" t="n">
-        <v>0.00175</v>
+        <v>0.00221</v>
       </c>
       <c r="E9" t="n">
-        <v>0.000481</v>
+        <v>0.000428</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>0.009719999999999999</v>
+        <v>0.0112</v>
       </c>
       <c r="H9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I9" s="1" t="inlineStr">
         <is>
-          <t>0/0/7</t>
+          <t>0/5/2</t>
         </is>
       </c>
       <c r="J9" s="1" t="inlineStr">
         <is>
-          <t>0/0/7</t>
+          <t>0/4/3</t>
         </is>
       </c>
       <c r="K9" s="1" t="inlineStr">
         <is>
-          <t>0/0/7</t>
+          <t>0/3/4</t>
         </is>
       </c>
       <c r="L9" s="1" t="inlineStr">
         <is>
-          <t>0/0/10</t>
+          <t>0/6/4</t>
         </is>
       </c>
       <c r="M9" t="n">
-        <v>77.97</v>
+        <v>60.29</v>
       </c>
       <c r="N9" s="1" t="inlineStr">
         <is>
-          <t>0.00E+00</t>
+          <t>1.04E-10</t>
         </is>
       </c>
     </row>
@@ -981,49 +981,49 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.012</v>
+        <v>0.009650000000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>0.00266</v>
+        <v>0.00219</v>
       </c>
       <c r="E10" t="n">
-        <v>0.000531</v>
+        <v>0.000527</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0133</v>
+        <v>0.011</v>
       </c>
       <c r="H10" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="I10" s="1" t="inlineStr">
         <is>
-          <t>0/7/0</t>
+          <t>0/2/5</t>
         </is>
       </c>
       <c r="J10" s="1" t="inlineStr">
         <is>
-          <t>0/7/0</t>
+          <t>0/3/4</t>
         </is>
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
-          <t>0/7/0</t>
+          <t>0/4/3</t>
         </is>
       </c>
       <c r="L10" s="1" t="inlineStr">
         <is>
-          <t>0/10/0</t>
+          <t>0/4/6</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>45.23</v>
+        <v>64.70999999999999</v>
       </c>
       <c r="N10" s="1" t="inlineStr">
         <is>
-          <t>6.35E-05</t>
+          <t>2.41E-12</t>
         </is>
       </c>
     </row>
@@ -1039,22 +1039,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.0138</v>
+        <v>0.0148</v>
       </c>
       <c r="D11" t="n">
-        <v>0.00315</v>
+        <v>0.00336</v>
       </c>
       <c r="E11" t="n">
-        <v>0.000634</v>
+        <v>0.0005730000000000001</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0157</v>
+        <v>0.0166</v>
       </c>
       <c r="H11" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="I11" s="1" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>17.81</v>
+        <v>16</v>
       </c>
       <c r="N11" s="1" t="inlineStr">
         <is>
@@ -1097,49 +1097,49 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.00247</v>
+        <v>0.00308</v>
       </c>
       <c r="D12" t="n">
-        <v>0.000514</v>
+        <v>0.000712</v>
       </c>
       <c r="E12" t="n">
-        <v>0.000577</v>
+        <v>0.0005730000000000001</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0.00302</v>
+        <v>0.0037</v>
       </c>
       <c r="H12" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I12" s="1" t="inlineStr">
         <is>
-          <t>0/1/0/0/6</t>
+          <t>1/0/0/3/3</t>
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>0/0/0/0/7</t>
+          <t>0/0/0/7/0</t>
         </is>
       </c>
       <c r="K12" s="1" t="inlineStr">
         <is>
-          <t>0/0/0/0/7</t>
+          <t>0/0/0/7/0</t>
         </is>
       </c>
       <c r="L12" s="1" t="inlineStr">
         <is>
-          <t>0/0/0/0/10</t>
+          <t>0/0/0/10/0</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>135.16</v>
+        <v>108.58</v>
       </c>
       <c r="N12" s="1" t="inlineStr">
         <is>
-          <t>0.00E+00</t>
+          <t>8.88E-16</t>
         </is>
       </c>
     </row>
@@ -1155,49 +1155,49 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.00401</v>
+        <v>0.00236</v>
       </c>
       <c r="D13" t="n">
-        <v>0.000851</v>
+        <v>0.000454</v>
       </c>
       <c r="E13" t="n">
-        <v>0.000569</v>
+        <v>0.000464</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0049</v>
+        <v>0.00272</v>
       </c>
       <c r="H13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I13" s="1" t="inlineStr">
         <is>
-          <t>0/0/1/6/0</t>
+          <t>0/0/0/4/3</t>
         </is>
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
-          <t>0/0/0/7/0</t>
+          <t>0/0/0/0/7</t>
         </is>
       </c>
       <c r="K13" s="1" t="inlineStr">
         <is>
-          <t>0/0/0/7/0</t>
+          <t>0/0/0/0/7</t>
         </is>
       </c>
       <c r="L13" s="1" t="inlineStr">
         <is>
-          <t>0/0/0/10/0</t>
+          <t>0/0/0/0/10</t>
         </is>
       </c>
       <c r="M13" t="n">
-        <v>108.16</v>
+        <v>133.77</v>
       </c>
       <c r="N13" s="1" t="inlineStr">
         <is>
-          <t>1.33E-15</t>
+          <t>0.00E+00</t>
         </is>
       </c>
     </row>
@@ -1213,26 +1213,26 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.0104</v>
+        <v>0.009339999999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00231</v>
+        <v>0.00213</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0004929999999999999</v>
+        <v>0.000527</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0124</v>
+        <v>0.0109</v>
       </c>
       <c r="H14" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>0/6/0/1/0</t>
+          <t>0/6/1/0/0</t>
         </is>
       </c>
       <c r="J14" s="1" t="inlineStr">
@@ -1251,11 +1251,11 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>50.19</v>
+        <v>51.65</v>
       </c>
       <c r="N14" s="1" t="inlineStr">
         <is>
-          <t>2.79E-03</t>
+          <t>1.79E-03</t>
         </is>
       </c>
     </row>
@@ -1271,22 +1271,22 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.00712</v>
+        <v>0.00469</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00151</v>
+        <v>0.0009700000000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>0.000439</v>
+        <v>0.000411</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0.008410000000000001</v>
+        <v>0.00571</v>
       </c>
       <c r="H15" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="I15" s="1" t="inlineStr">
         <is>
@@ -1309,11 +1309,11 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>80.39</v>
+        <v>79.97</v>
       </c>
       <c r="N15" s="1" t="inlineStr">
         <is>
-          <t>2.29E-08</t>
+          <t>2.74E-08</t>
         </is>
       </c>
     </row>
@@ -1329,45 +1329,45 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.033</v>
+        <v>0.0375</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00755</v>
+        <v>0.008829999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>0.000664</v>
+        <v>0.000572</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0369</v>
+        <v>0.0412</v>
       </c>
       <c r="H16" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I16" s="1" t="inlineStr">
         <is>
+          <t>6/1/0/0/0</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
           <t>7/0/0/0/0</t>
         </is>
       </c>
-      <c r="J16" s="1" t="inlineStr">
+      <c r="K16" s="1" t="inlineStr">
         <is>
           <t>7/0/0/0/0</t>
         </is>
       </c>
-      <c r="K16" s="1" t="inlineStr">
-        <is>
-          <t>7/0/0/0/0</t>
-        </is>
-      </c>
       <c r="L16" s="1" t="inlineStr">
         <is>
           <t>10/0/0/0/0</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>16.1</v>
+        <v>16.03</v>
       </c>
       <c r="N16" s="1" t="inlineStr">
         <is>
@@ -1387,22 +1387,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.000537</v>
+        <v>0.00052</v>
       </c>
       <c r="D17" t="n">
-        <v>3.91e-05</v>
+        <v>3.15e-05</v>
       </c>
       <c r="E17" t="n">
-        <v>0.000464</v>
+        <v>0.000477</v>
       </c>
       <c r="F17" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G17" t="n">
-        <v>0.000618</v>
+        <v>0.000611</v>
       </c>
       <c r="H17" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="I17" s="1" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>132.74</v>
+        <v>133.9</v>
       </c>
       <c r="N17" s="1" t="inlineStr">
         <is>
@@ -1445,26 +1445,26 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.000754</v>
+        <v>0.000932</v>
       </c>
       <c r="D18" t="n">
-        <v>9.98e-05</v>
+        <v>0.000121</v>
       </c>
       <c r="E18" t="n">
-        <v>0.000416</v>
+        <v>0.000426</v>
       </c>
       <c r="F18" t="n">
         <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>0.000969</v>
+        <v>0.00109</v>
       </c>
       <c r="H18" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="I18" s="1" t="inlineStr">
         <is>
-          <t>0/0/0/6/1</t>
+          <t>0/0/0/7/0</t>
         </is>
       </c>
       <c r="J18" s="1" t="inlineStr">
@@ -1483,11 +1483,11 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>112.35</v>
+        <v>110</v>
       </c>
       <c r="N18" s="1" t="inlineStr">
         <is>
-          <t>4.44E-16</t>
+          <t>1.33E-15</t>
         </is>
       </c>
     </row>
@@ -1503,26 +1503,26 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.0027</v>
+        <v>0.00219</v>
       </c>
       <c r="D19" t="n">
-        <v>0.000521</v>
+        <v>0.000506</v>
       </c>
       <c r="E19" t="n">
-        <v>0.000455</v>
+        <v>0.000413</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0.00335</v>
+        <v>0.00305</v>
       </c>
       <c r="H19" t="n">
         <v>31</v>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>0/0/6/1/0</t>
+          <t>0/0/6/0/1</t>
         </is>
       </c>
       <c r="J19" s="1" t="inlineStr">
@@ -1541,11 +1541,11 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>81.87</v>
+        <v>83.06</v>
       </c>
       <c r="N19" s="1" t="inlineStr">
         <is>
-          <t>2.69E-08</t>
+          <t>1.46E-08</t>
         </is>
       </c>
     </row>
@@ -1561,22 +1561,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.0213</v>
+        <v>0.0202</v>
       </c>
       <c r="D20" t="n">
-        <v>0.00476</v>
+        <v>0.00468</v>
       </c>
       <c r="E20" t="n">
-        <v>0.000466</v>
+        <v>0.000427</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.024</v>
+        <v>0.0232</v>
       </c>
       <c r="H20" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I20" s="1" t="inlineStr">
         <is>
@@ -1619,22 +1619,22 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.0318</v>
+        <v>0.0332</v>
       </c>
       <c r="D21" t="n">
-        <v>0.00721</v>
+        <v>0.00774</v>
       </c>
       <c r="E21" t="n">
-        <v>0.00087</v>
+        <v>0.000739</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0.035</v>
+        <v>0.0368</v>
       </c>
       <c r="H21" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I21" s="1" t="inlineStr">
         <is>
@@ -1680,19 +1680,19 @@
         <v>0.0013</v>
       </c>
       <c r="D22" t="n">
-        <v>0.000149</v>
+        <v>0.000141</v>
       </c>
       <c r="E22" t="n">
-        <v>0.000601</v>
+        <v>0.000613</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0.00149</v>
+        <v>0.00145</v>
       </c>
       <c r="H22" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="I22" s="1" t="inlineStr">
         <is>
@@ -1715,11 +1715,11 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>81.34999999999999</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="N22" s="1" t="inlineStr">
         <is>
-          <t>8.64E-09</t>
+          <t>7.94E-09</t>
         </is>
       </c>
     </row>
@@ -1735,19 +1735,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2.01e-05</v>
+        <v>2.18e-05</v>
       </c>
       <c r="D23" t="n">
-        <v>2.16e-05</v>
+        <v>2.04e-05</v>
       </c>
       <c r="E23" t="n">
-        <v>5.59e-09</v>
+        <v>2.31e-06</v>
       </c>
       <c r="F23" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G23" t="n">
-        <v>9.02e-05</v>
+        <v>7.889999999999999e-05</v>
       </c>
       <c r="H23" t="n">
         <v>8</v>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>105.35</v>
+        <v>105.61</v>
       </c>
       <c r="N23" s="1" t="inlineStr">
         <is>
@@ -1793,19 +1793,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.00483</v>
+        <v>0.00484</v>
       </c>
       <c r="D24" t="n">
-        <v>0.00219</v>
+        <v>0.00223</v>
       </c>
       <c r="E24" t="n">
-        <v>0.000325</v>
+        <v>0.000326</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.00838</v>
       </c>
       <c r="H24" t="n">
         <v>26</v>
@@ -1831,11 +1831,11 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>35.1</v>
+        <v>35.48</v>
       </c>
       <c r="N24" s="1" t="inlineStr">
         <is>
-          <t>4.50E-01</t>
+          <t>4.00E-01</t>
         </is>
       </c>
     </row>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.00503</v>
+        <v>0.00508</v>
       </c>
       <c r="D25" t="n">
-        <v>0.00137</v>
+        <v>0.00131</v>
       </c>
       <c r="E25" t="n">
-        <v>0.000859</v>
+        <v>0.0009210000000000001</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0.00697</v>
+        <v>0.00703</v>
       </c>
       <c r="H25" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I25" s="1" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>28.19</v>
+        <v>27.81</v>
       </c>
       <c r="N25" s="1" t="inlineStr">
         <is>

</xml_diff>